<commit_message>
📅 Quitar diciembre (desde enero) + Excel 564 transacciones
</commit_message>
<xml_diff>
--- a/Gastos_Richard_2026.xlsx
+++ b/Gastos_Richard_2026.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transacciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Transacciones'!$A$1:$H$567</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Transacciones'!$A$1:$H$565</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="5">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>50756.22</v>
+        <v>50566.22</v>
       </c>
     </row>
     <row r="6">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>31906.22</v>
+        <v>31716.22</v>
       </c>
     </row>
     <row r="9">
@@ -590,10 +590,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>10886.27</v>
+        <v>10796.27</v>
       </c>
     </row>
     <row r="13">
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>10637.28</v>
+        <v>10537.28</v>
       </c>
     </row>
     <row r="14">
@@ -733,10 +733,10 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>50756.22</v>
+        <v>50566.22</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H568"/>
+  <dimension ref="A1:H566"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21110,89 +21110,17 @@
       </c>
     </row>
     <row r="566">
-      <c r="A566" s="9" t="inlineStr">
-        <is>
-          <t>12/26/2026</t>
-        </is>
-      </c>
-      <c r="B566" s="9" t="inlineStr">
-        <is>
-          <t>Depósito EFT Paypal</t>
-        </is>
-      </c>
-      <c r="C566" s="9" t="inlineStr">
-        <is>
-          <t>Depósito EFT Paypal</t>
-        </is>
-      </c>
-      <c r="D566" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="E566" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F566" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="G566" s="11" t="inlineStr">
-        <is>
-          <t>Transferencia</t>
-        </is>
-      </c>
-      <c r="H566" s="9" t="inlineStr">
-        <is>
-          <t>Cuenta Cheques 243-095208</t>
-        </is>
-      </c>
-    </row>
-    <row r="567">
-      <c r="A567" s="9" t="inlineStr">
-        <is>
-          <t>12/26/2026</t>
-        </is>
-      </c>
-      <c r="B567" s="9" t="inlineStr">
-        <is>
-          <t>Pago EFT Paypal Inst xfer SIRILED</t>
-        </is>
-      </c>
-      <c r="C567" s="9" t="inlineStr">
-        <is>
-          <t>Pago EFT Paypal Inst xfer SIRILED</t>
-        </is>
-      </c>
-      <c r="D567" s="10" t="n">
-        <v>90</v>
-      </c>
-      <c r="E567" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F567" s="10" t="n">
-        <v>90</v>
-      </c>
-      <c r="G567" s="11" t="inlineStr">
-        <is>
-          <t>Pago EFT</t>
-        </is>
-      </c>
-      <c r="H567" s="9" t="inlineStr">
-        <is>
-          <t>Cuenta Cheques 243-095208</t>
-        </is>
-      </c>
-    </row>
-    <row r="568">
-      <c r="E568" s="2" t="inlineStr">
+      <c r="E566" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F568" s="12" t="n">
-        <v>50756.22</v>
+      <c r="F566" s="12" t="n">
+        <v>50566.22</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H567"/>
+  <autoFilter ref="A1:H565"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>